<commit_message>
Add magazine/article-1 import artifacts + project config
URL list, regenerated import report for magazine/article-1, and
.claude-plugin project/sites config from handover doc generation.
(Page content lives in Document Authoring, already published.)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>_reportFile</t>
   </si>
@@ -56,6 +56,18 @@
   </si>
   <si>
     <t>https://wknd-trendsetters.site/about-us</t>
+  </si>
+  <si>
+    <t>magazine/article-1.report.json</t>
+  </si>
+  <si>
+    <t>magazine/article-1</t>
+  </si>
+  <si>
+    <t>2026-08-05T15:11:57.637Z</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/magazine/article-1</t>
   </si>
 </sst>
 </file>
@@ -444,16 +456,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="41" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -506,6 +517,32 @@
       </c>
       <c r="H2" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bulk import magazine/article-1..3 artifacts
URL list + import reports for the 3 magazine pages (content published
to Document Authoring). Reused the about-us import bundle.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="27">
   <si>
     <t>_reportFile</t>
   </si>
@@ -64,10 +64,34 @@
     <t>magazine/article-1</t>
   </si>
   <si>
-    <t>2026-08-05T15:11:57.637Z</t>
+    <t>2026-08-05T15:26:14.452Z</t>
   </si>
   <si>
     <t>https://wknd-trendsetters.site/magazine/article-1</t>
+  </si>
+  <si>
+    <t>magazine/article-2.report.json</t>
+  </si>
+  <si>
+    <t>magazine/article-2</t>
+  </si>
+  <si>
+    <t>2026-08-05T15:26:20.677Z</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/magazine/article-2</t>
+  </si>
+  <si>
+    <t>magazine/article-3.report.json</t>
+  </si>
+  <si>
+    <t>magazine/article-3</t>
+  </si>
+  <si>
+    <t>2026-08-05T15:26:27.367Z</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/magazine/article-3</t>
   </si>
 </sst>
 </file>
@@ -456,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -545,6 +569,58 @@
         <v>18</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>